<commit_message>
feat(producao): importações aceitam a planilha única do gestor (local 1 / local 5 e 'pedido ttl' em unidades), além do formato do ERP
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/automatizando processos_/modelo-produtos-preenchido.xlsx
+++ b/automatizando processos_/modelo-produtos-preenchido.xlsx
@@ -598,14 +598,14 @@
         <v>3651</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="H2" s="4">
         <f>F2+G2</f>
         <v/>
       </c>
       <c r="I2" s="5" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="J2" s="6">
         <f>H2-I2</f>
@@ -869,7 +869,7 @@
         <v/>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="J8" s="6">
         <f>H8-I8</f>
@@ -1082,14 +1082,14 @@
         <v>538</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="H13" s="10">
         <f>F13+G13</f>
         <v/>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0</v>
+        <v>720</v>
       </c>
       <c r="J13" s="11">
         <f>H13-I13</f>
@@ -1177,7 +1177,7 @@
         <v/>
       </c>
       <c r="I15" s="5" t="n">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="J15" s="11">
         <f>H15-I15</f>
@@ -1265,7 +1265,7 @@
         <v/>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0</v>
+        <v>576</v>
       </c>
       <c r="J17" s="11">
         <f>H17-I17</f>
@@ -1566,14 +1566,14 @@
         <v>470</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="H24" s="4">
         <f>F24+G24</f>
         <v/>
       </c>
       <c r="I24" s="5" t="n">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="J24" s="6">
         <f>H24-I24</f>
@@ -1617,7 +1617,7 @@
         <v/>
       </c>
       <c r="I25" s="5" t="n">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="J25" s="11">
         <f>H25-I25</f>
@@ -1698,14 +1698,14 @@
         <v>3232</v>
       </c>
       <c r="G27" s="10" t="n">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="H27" s="10">
         <f>F27+G27</f>
         <v/>
       </c>
       <c r="I27" s="5" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="J27" s="11">
         <f>H27-I27</f>
@@ -1925,7 +1925,7 @@
         <v/>
       </c>
       <c r="I32" s="5" t="n">
-        <v>0</v>
+        <v>576</v>
       </c>
       <c r="J32" s="6">
         <f>H32-I32</f>
@@ -2321,7 +2321,7 @@
         <v/>
       </c>
       <c r="I41" s="5" t="n">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="J41" s="11">
         <f>H41-I41</f>
@@ -2365,7 +2365,7 @@
         <v/>
       </c>
       <c r="I42" s="5" t="n">
-        <v>0</v>
+        <v>288</v>
       </c>
       <c r="J42" s="6">
         <f>H42-I42</f>
@@ -2497,7 +2497,7 @@
         <v/>
       </c>
       <c r="I45" s="5" t="n">
-        <v>0</v>
+        <v>384</v>
       </c>
       <c r="J45" s="11">
         <f>H45-I45</f>

</xml_diff>

<commit_message>
feat(producao): tags de referência para filtrar cadastro e necessidade; Gr de uso sai da tabela de cadastro (segue no cálculo e em Produzir)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/automatizando processos_/modelo-produtos-preenchido.xlsx
+++ b/automatizando processos_/modelo-produtos-preenchido.xlsx
@@ -604,9 +604,7 @@
         <f>F2+G2</f>
         <v/>
       </c>
-      <c r="I2" s="5" t="n">
-        <v>480</v>
-      </c>
+      <c r="I2" s="5" t="n"/>
       <c r="J2" s="6">
         <f>H2-I2</f>
         <v/>
@@ -648,9 +646,7 @@
         <f>F3+G3</f>
         <v/>
       </c>
-      <c r="I3" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I3" s="5" t="n"/>
       <c r="J3" s="11">
         <f>H3-I3</f>
         <v/>
@@ -692,9 +688,7 @@
         <f>F4+G4</f>
         <v/>
       </c>
-      <c r="I4" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I4" s="5" t="n"/>
       <c r="J4" s="6">
         <f>H4-I4</f>
         <v/>
@@ -736,9 +730,7 @@
         <f>F5+G5</f>
         <v/>
       </c>
-      <c r="I5" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I5" s="5" t="n"/>
       <c r="J5" s="11">
         <f>H5-I5</f>
         <v/>
@@ -780,9 +772,7 @@
         <f>F6+G6</f>
         <v/>
       </c>
-      <c r="I6" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I6" s="5" t="n"/>
       <c r="J6" s="6">
         <f>H6-I6</f>
         <v/>
@@ -824,9 +814,7 @@
         <f>F7+G7</f>
         <v/>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I7" s="5" t="n"/>
       <c r="J7" s="11">
         <f>H7-I7</f>
         <v/>
@@ -868,9 +856,7 @@
         <f>F8+G8</f>
         <v/>
       </c>
-      <c r="I8" s="5" t="n">
-        <v>960</v>
-      </c>
+      <c r="I8" s="5" t="n"/>
       <c r="J8" s="6">
         <f>H8-I8</f>
         <v/>
@@ -912,9 +898,7 @@
         <f>F9+G9</f>
         <v/>
       </c>
-      <c r="I9" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I9" s="5" t="n"/>
       <c r="J9" s="11">
         <f>H9-I9</f>
         <v/>
@@ -956,9 +940,7 @@
         <f>F10+G10</f>
         <v/>
       </c>
-      <c r="I10" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I10" s="5" t="n"/>
       <c r="J10" s="6">
         <f>H10-I10</f>
         <v/>
@@ -1000,9 +982,7 @@
         <f>F11+G11</f>
         <v/>
       </c>
-      <c r="I11" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I11" s="5" t="n"/>
       <c r="J11" s="11">
         <f>H11-I11</f>
         <v/>
@@ -1044,9 +1024,7 @@
         <f>F12+G12</f>
         <v/>
       </c>
-      <c r="I12" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I12" s="5" t="n"/>
       <c r="J12" s="6">
         <f>H12-I12</f>
         <v/>
@@ -1088,9 +1066,7 @@
         <f>F13+G13</f>
         <v/>
       </c>
-      <c r="I13" s="5" t="n">
-        <v>720</v>
-      </c>
+      <c r="I13" s="5" t="n"/>
       <c r="J13" s="11">
         <f>H13-I13</f>
         <v/>
@@ -1132,9 +1108,7 @@
         <f>F14+G14</f>
         <v/>
       </c>
-      <c r="I14" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I14" s="5" t="n"/>
       <c r="J14" s="6">
         <f>H14-I14</f>
         <v/>
@@ -1176,9 +1150,7 @@
         <f>F15+G15</f>
         <v/>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>1200</v>
-      </c>
+      <c r="I15" s="5" t="n"/>
       <c r="J15" s="11">
         <f>H15-I15</f>
         <v/>
@@ -1220,9 +1192,7 @@
         <f>F16+G16</f>
         <v/>
       </c>
-      <c r="I16" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I16" s="5" t="n"/>
       <c r="J16" s="6">
         <f>H16-I16</f>
         <v/>
@@ -1264,9 +1234,7 @@
         <f>F17+G17</f>
         <v/>
       </c>
-      <c r="I17" s="5" t="n">
-        <v>576</v>
-      </c>
+      <c r="I17" s="5" t="n"/>
       <c r="J17" s="11">
         <f>H17-I17</f>
         <v/>
@@ -1308,9 +1276,7 @@
         <f>F18+G18</f>
         <v/>
       </c>
-      <c r="I18" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I18" s="5" t="n"/>
       <c r="J18" s="6">
         <f>H18-I18</f>
         <v/>
@@ -1352,9 +1318,7 @@
         <f>F19+G19</f>
         <v/>
       </c>
-      <c r="I19" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I19" s="5" t="n"/>
       <c r="J19" s="11">
         <f>H19-I19</f>
         <v/>
@@ -1396,9 +1360,7 @@
         <f>F20+G20</f>
         <v/>
       </c>
-      <c r="I20" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I20" s="5" t="n"/>
       <c r="J20" s="6">
         <f>H20-I20</f>
         <v/>
@@ -1440,9 +1402,7 @@
         <f>F21+G21</f>
         <v/>
       </c>
-      <c r="I21" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I21" s="5" t="n"/>
       <c r="J21" s="11">
         <f>H21-I21</f>
         <v/>
@@ -1484,9 +1444,7 @@
         <f>F22+G22</f>
         <v/>
       </c>
-      <c r="I22" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I22" s="5" t="n"/>
       <c r="J22" s="6">
         <f>H22-I22</f>
         <v/>
@@ -1528,9 +1486,7 @@
         <f>F23+G23</f>
         <v/>
       </c>
-      <c r="I23" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I23" s="5" t="n"/>
       <c r="J23" s="11">
         <f>H23-I23</f>
         <v/>
@@ -1572,9 +1528,7 @@
         <f>F24+G24</f>
         <v/>
       </c>
-      <c r="I24" s="5" t="n">
-        <v>1440</v>
-      </c>
+      <c r="I24" s="5" t="n"/>
       <c r="J24" s="6">
         <f>H24-I24</f>
         <v/>
@@ -1616,9 +1570,7 @@
         <f>F25+G25</f>
         <v/>
       </c>
-      <c r="I25" s="5" t="n">
-        <v>960</v>
-      </c>
+      <c r="I25" s="5" t="n"/>
       <c r="J25" s="11">
         <f>H25-I25</f>
         <v/>
@@ -1660,9 +1612,7 @@
         <f>F26+G26</f>
         <v/>
       </c>
-      <c r="I26" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I26" s="5" t="n"/>
       <c r="J26" s="6">
         <f>H26-I26</f>
         <v/>
@@ -1704,9 +1654,7 @@
         <f>F27+G27</f>
         <v/>
       </c>
-      <c r="I27" s="5" t="n">
-        <v>240</v>
-      </c>
+      <c r="I27" s="5" t="n"/>
       <c r="J27" s="11">
         <f>H27-I27</f>
         <v/>
@@ -1748,9 +1696,7 @@
         <f>F28+G28</f>
         <v/>
       </c>
-      <c r="I28" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I28" s="5" t="n"/>
       <c r="J28" s="6">
         <f>H28-I28</f>
         <v/>
@@ -1792,9 +1738,7 @@
         <f>F29+G29</f>
         <v/>
       </c>
-      <c r="I29" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I29" s="5" t="n"/>
       <c r="J29" s="11">
         <f>H29-I29</f>
         <v/>
@@ -1836,9 +1780,7 @@
         <f>F30+G30</f>
         <v/>
       </c>
-      <c r="I30" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I30" s="5" t="n"/>
       <c r="J30" s="6">
         <f>H30-I30</f>
         <v/>
@@ -1880,9 +1822,7 @@
         <f>F31+G31</f>
         <v/>
       </c>
-      <c r="I31" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I31" s="5" t="n"/>
       <c r="J31" s="11">
         <f>H31-I31</f>
         <v/>
@@ -1924,9 +1864,7 @@
         <f>F32+G32</f>
         <v/>
       </c>
-      <c r="I32" s="5" t="n">
-        <v>576</v>
-      </c>
+      <c r="I32" s="5" t="n"/>
       <c r="J32" s="6">
         <f>H32-I32</f>
         <v/>
@@ -1968,9 +1906,7 @@
         <f>F33+G33</f>
         <v/>
       </c>
-      <c r="I33" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I33" s="5" t="n"/>
       <c r="J33" s="11">
         <f>H33-I33</f>
         <v/>
@@ -2012,9 +1948,7 @@
         <f>F34+G34</f>
         <v/>
       </c>
-      <c r="I34" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I34" s="5" t="n"/>
       <c r="J34" s="6">
         <f>H34-I34</f>
         <v/>
@@ -2056,9 +1990,7 @@
         <f>F35+G35</f>
         <v/>
       </c>
-      <c r="I35" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I35" s="5" t="n"/>
       <c r="J35" s="11">
         <f>H35-I35</f>
         <v/>
@@ -2100,9 +2032,7 @@
         <f>F36+G36</f>
         <v/>
       </c>
-      <c r="I36" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I36" s="5" t="n"/>
       <c r="J36" s="6">
         <f>H36-I36</f>
         <v/>
@@ -2144,9 +2074,7 @@
         <f>F37+G37</f>
         <v/>
       </c>
-      <c r="I37" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I37" s="5" t="n"/>
       <c r="J37" s="11">
         <f>H37-I37</f>
         <v/>
@@ -2188,9 +2116,7 @@
         <f>F38+G38</f>
         <v/>
       </c>
-      <c r="I38" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I38" s="5" t="n"/>
       <c r="J38" s="6">
         <f>H38-I38</f>
         <v/>
@@ -2232,9 +2158,7 @@
         <f>F39+G39</f>
         <v/>
       </c>
-      <c r="I39" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I39" s="5" t="n"/>
       <c r="J39" s="11">
         <f>H39-I39</f>
         <v/>
@@ -2276,9 +2200,7 @@
         <f>F40+G40</f>
         <v/>
       </c>
-      <c r="I40" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I40" s="5" t="n"/>
       <c r="J40" s="6">
         <f>H40-I40</f>
         <v/>
@@ -2320,9 +2242,7 @@
         <f>F41+G41</f>
         <v/>
       </c>
-      <c r="I41" s="5" t="n">
-        <v>240</v>
-      </c>
+      <c r="I41" s="5" t="n"/>
       <c r="J41" s="11">
         <f>H41-I41</f>
         <v/>
@@ -2364,9 +2284,7 @@
         <f>F42+G42</f>
         <v/>
       </c>
-      <c r="I42" s="5" t="n">
-        <v>288</v>
-      </c>
+      <c r="I42" s="5" t="n"/>
       <c r="J42" s="6">
         <f>H42-I42</f>
         <v/>
@@ -2408,9 +2326,7 @@
         <f>F43+G43</f>
         <v/>
       </c>
-      <c r="I43" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I43" s="5" t="n"/>
       <c r="J43" s="11">
         <f>H43-I43</f>
         <v/>
@@ -2452,9 +2368,7 @@
         <f>F44+G44</f>
         <v/>
       </c>
-      <c r="I44" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I44" s="5" t="n"/>
       <c r="J44" s="6">
         <f>H44-I44</f>
         <v/>
@@ -2496,9 +2410,7 @@
         <f>F45+G45</f>
         <v/>
       </c>
-      <c r="I45" s="5" t="n">
-        <v>384</v>
-      </c>
+      <c r="I45" s="5" t="n"/>
       <c r="J45" s="11">
         <f>H45-I45</f>
         <v/>
@@ -2540,9 +2452,7 @@
         <f>F46+G46</f>
         <v/>
       </c>
-      <c r="I46" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I46" s="5" t="n"/>
       <c r="J46" s="6">
         <f>H46-I46</f>
         <v/>
@@ -2591,7 +2501,7 @@
     <row r="49">
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>Coluna 'pedido ttl' (amarela): preencher com o total pedido pelas lojas. As demais calculam sozinhas: estoque disponível = local 1 + local 5; produzir = estoque − pedido (negativo = falta produzir); quilos = produzir × peso para produção.</t>
+          <t>Este arquivo é o CADASTRO + ESTOQUE: use nos botões Importar cadastro e Importar estoque atual. A coluna 'pedido ttl' fica vazia — o pedido vem do PDF do cliente, pelo botão Importar pedido. As colunas de cálculo (estoque disponível, produzir, quilos) são só conferência no Excel.</t>
         </is>
       </c>
     </row>

</xml_diff>